<commit_message>
Updated Economy and Fixed Bugs
1. Updated economy from level 1-30 and first testing is done.
2. Removed wrong path follow and some zig-zag movements on nurse's paths.
3. Added dynamic machine and worker speed on the basis of duration upgrade of stations (only those having workers behind).
</commit_message>
<xml_diff>
--- a/Assets/Resources/HappyDiner/Happy Hospital Formatted Economy v2.xlsx
+++ b/Assets/Resources/HappyDiner/Happy Hospital Formatted Economy v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Unity Projects\Git\Hospitalscape\Assets\Resources\HappyDiner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B57E6D9-4C43-44E4-84C1-F466D9969D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD09ED6-517A-4C95-B9DE-2841631C092B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3244,7 +3244,9 @@
         <v>80</v>
       </c>
       <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="H2" s="3">
+        <v>3</v>
+      </c>
       <c r="I2" s="3" t="b">
         <v>0</v>
       </c>
@@ -3454,7 +3456,9 @@
         <v>235</v>
       </c>
       <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="H4" s="3">
+        <v>5</v>
+      </c>
       <c r="I4" s="3" t="b">
         <v>0</v>
       </c>
@@ -4531,7 +4535,7 @@
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E12" s="3">
         <v>7</v>

</xml_diff>